<commit_message>
feat(F-NAR-019): ATOM-AUT.AFF.001-07 La plume d'Aniss
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.001-07.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.001-07.xlsx
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Aniss veut l'oiseau du bois. Le chapeau tombe, le doudou est sur la chaise. Il range, marche, une plume lui chatouille le doigt.</t>
+          <t>Une ombre d'arbre entre dans la cuisine. Sur la vitre, un grain de pin colle. Aniss veut la plume grise sous l'arbre, maintenant, dans sa boîte. Il pousse tout dans le sac : le zip mord le chapeau. Il refuse de forcer, range une chose puis l'autre, glisse le grain. Sur le chemin, une branche barre le pas. Il refuse de foncer. Sous l'arbre, le grain de pin brille sur la plume.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Une branche frotte le chemin du bois. Les aiguilles de pin sentent le chaud. Une tartine croustille sur l'assiette. Ça sent le beurre. Un oiseau chante déjà dehors. Les crochets cliquettent un peu. Le tapis de l'entrée est un peu rêche. Une miette tombe près de la tasse. Papa verse un peu d'eau. L'eau fait un bruit clair. La tartine a un bord doré. Elle croustille, papa. Une dernière bouchée ? Oui. Aniss, tu entends l'oiseau ? Oui, je veux le voir dans le bois. On y va, avec le sac. En ce moment, Aniss s'accroupit. Le sac est posé contre la porte. Il est un peu froid. Le sac est bleu. Prends de l'eau, le chemin est long. Aniss prend la gourde. Elle est fraîche. Il la met dans le sac. Le chapeau aussi, les branches piquent. Aniss prend le chapeau. Le bord est un peu souple. Le chapeau glisse par terre. Il est tombé. Tu le ramasses, puis dans le sac. Aniss ramasse le chapeau. Il le met dans le sac. Et le doudou ? Le doudou n'est pas près des chaussures. Regarde la chaise de la cuisine.</t>
+          <t>Une ombre d'arbre entre dans la cuisine. Elle glisse sur la nappe, puis la tasse. Aniss lève les yeux vers la fenêtre. Les planches sentent la résine, tiède. Pourtant, un détail paraît nouveau. Une pomme de pin s'est ouverte sur le rebord. Un grain de pin colle à la vitre. Il est brun, collant, et il sent le bois. Il est tout petit, papa. C'est un grain tombé du pin. Le grain brille comme un bout d'étoile. Dehors, le grand arbre penche vers le chemin. Une plume grise tremble dans l'herbe, au loin. Je veux cette plume, maintenant ! Aniss, tu vois l'arbre ? Oui, papa. Elle m'attend. On y va, avec le sac. En ce moment, Aniss saisit le sac bleu. Le tissu gratte sous ses doigts. Prends de l'eau, pour le chemin. Aniss prend la gourde fraîche. Le bouchon est froid sous le doigt. Le chapeau aussi, les branches piquent. Aniss prend le chapeau souple. Le bord plie un peu, dans sa main. Et ma boîte à plumes ? La boîte de bois attend sur le banc. Je mets tout, d'un coup ! Il pousse gourde, chapeau et boîte. La boîte tape le fond, trop vite. Le zip mord le bord du chapeau. Ça reste coincé ! Le sourire d'Aniss disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu regardes le zip ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Une branche frotte le chemin du bois. Les aiguilles de pin sentent le chaud. Une tartine croustille sur l'assiette. Ça sent le beurre. Un oiseau chante déjà dehors. Les crochets cliquettent un peu. Le tapis de l'entrée est un peu rêche. Une miette tombe près de la tasse. Papa verse un peu d'eau. L'eau fait un bruit clair. La tartine a un bord doré. Elle croustille, papa. Une dernière bouchée ? Oui. Aniss, tu entends l'oiseau ? Oui, je veux le voir dans le bois. On y va, avec le sac. En ce moment, Aniss s'accroupit. Le sac est posé contre la porte. Il est un peu froid. Le sac est bleu. Prends de l'eau, le chemin est long. Aniss prend la gourde. Elle est fraîche. Il la met dans le sac. Le chapeau aussi, les branches piquent. Aniss prend le chapeau. Le bord est un peu souple. Le chapeau glisse par terre. Il est tombé. Tu le ramasses, puis dans le sac. Aniss ramasse le chapeau. Il le met dans le sac. Et le doudou ? Le doudou n'est pas près des chaussures. Regarde la chaise de la cuisine.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une ombre d'arbre entre dans la cuisine. Elle glisse sur la nappe, puis la tasse. Aniss lève les yeux vers la fenêtre. Les planches sentent la résine, tiède. Pourtant, un détail paraît nouveau. Une pomme de pin s'est ouverte sur le rebord. Un &lt;emphasis level="moderate"&gt;grain de pin&lt;/emphasis&gt; colle à la vitre. Il est brun, collant, et il sent le bois. Il est tout petit, papa. C'est un grain tombé du pin. Le grain brille comme un bout d'étoile. Dehors, le grand arbre penche vers le chemin. Une plume grise tremble dans l'herbe, au loin. Je veux cette plume, maintenant ! Aniss, tu vois l'arbre ? Oui, papa. Elle m'attend. On y va, avec le sac. En ce moment, Aniss saisit le sac bleu. Le tissu gratte sous ses doigts. Prends de l'eau, pour le chemin. Aniss prend la gourde fraîche. Le bouchon est froid sous le doigt. Le chapeau aussi, les branches piquent. Aniss prend le chapeau souple. Le bord plie un peu, dans sa main. Et ma boîte à plumes ? La boîte de bois attend sur le banc. Je mets tout, d'un coup ! Il pousse gourde, chapeau et boîte. La boîte tape le fond, trop vite. Le zip mord le bord du chapeau. Ça reste coincé ! Le sourire d'Aniss disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu regardes le zip ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Clara va au parc avec papa. Papa pose le &lt;emphasis&gt;sac&lt;/emphasis&gt; ouvert. Papa dit : on met la gourde. On met le chapeau. On met le doudou. C'est ce que l'adulte a dit. Clara prend la gourde. Elle la met dans le sac. Le sac est bleu. Clara prend le chapeau. Elle le met dans le sac. Elle prend le doudou. Elle le met dans le sac. Papa dit : tu as mis ce que l'adulte a dit. Clara ferme le sac. Elle le porte. À l'entrée, elle vérifie. Gourde, chapeau, doudou. Tout est dans le sac. Papa sourit. Clara a préparé son sac. [pause]</t>
+          <t>Une ombre d'arbre entre dans la cuisine. Elle glisse sur la nappe, puis la tasse. Aniss lève les yeux vers la fenêtre. Les planches sentent la résine, tiède. Pourtant, un détail paraît nouveau. Une pomme de pin s'est ouverte sur le rebord. Un &lt;emphasis&gt;grain de pin&lt;/emphasis&gt; colle à la vitre. Il est brun, collant, et il sent le bois. Il est tout petit, papa. C'est un grain tombé du pin. Le grain brille comme un bout d'étoile. Dehors, le grand arbre penche vers le chemin. Une plume grise tremble dans l'herbe, au loin. Je veux cette plume, maintenant ! Aniss, tu vois l'arbre ? Oui, papa. Elle m'attend. On y va, avec le sac. En ce moment, Aniss saisit le sac bleu. Le tissu gratte sous ses doigts. Prends de l'eau, pour le chemin. Aniss prend la gourde fraîche. Le bouchon est froid sous le doigt. Le chapeau aussi, les branches piquent. Aniss prend le chapeau souple. Le bord plie un peu, dans sa main. Et ma boîte à plumes ? La boîte de bois attend sur le banc. Je mets tout, d'un coup ! Il pousse gourde, chapeau et boîte. La boîte tape le fond, trop vite. Le zip mord le bord du chapeau. Ça reste coincé ! Le sourire d'Aniss disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu regardes le zip ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>sac</t>
+          <t>grain de pin</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,50 +1321,54 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_la_plume_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Une branche frotte le chemin du bois.
-narrateur|Les aiguilles de pin sentent le chaud.
-narrateur|Une tartine croustille sur l'assiette.
-narrateur|Ça sent le beurre.
-narrateur|Un oiseau chante déjà dehors.
-narrateur|Les crochets cliquettent un peu.
-narrateur|Le tapis de l'entrée est un peu rêche.
-narrateur|Une miette tombe près de la tasse.
-narrateur|Papa verse un peu d'eau.
-narrateur|L'eau fait un bruit clair.
-narrateur|La tartine a un bord doré.
-enfant-m|Elle croustille, papa.
-papa|Une dernière bouchée ?
-enfant-m|Oui.
-papa|Aniss, tu entends l'oiseau ?
-enfant-m|Oui, je veux le voir dans le bois.
+          <t>narrateur|Une ombre d'arbre entre dans la cuisine.
+narrateur|Elle glisse sur la nappe, puis la tasse.
+narrateur|Aniss lève les yeux vers la fenêtre.
+narrateur|Les planches sentent la résine, tiède.
+narrateur|Pourtant, un détail paraît nouveau.
+narrateur|Une pomme de pin s'est ouverte sur le rebord.
+narrateur|Un grain de pin colle à la vitre.
+narrateur|Il est brun, collant, et il sent le bois.
+enfant-m|Il est tout petit, papa.
+papa|C'est un grain tombé du pin.
+narrateur|Le grain brille comme un bout d'étoile.
+narrateur|Dehors, le grand arbre penche vers le chemin.
+narrateur|Une plume grise tremble dans l'herbe, au loin.
+enfant-m|Je veux cette plume, maintenant !
+papa|Aniss, tu vois l'arbre ?
+enfant-m|Oui, papa.
+enfant-m|Elle m'attend.
 papa|On y va, avec le sac.
-narrateur|En ce moment, Aniss s'accroupit.
-narrateur|Le sac est posé contre la porte.
-narrateur|Il est un peu froid.
-narrateur|Le sac est bleu.
-papa|Prends de l'eau, le chemin est long.
-narrateur|Aniss prend la gourde.
-narrateur|Elle est fraîche.
-narrateur|Il la met dans le sac.
+narrateur|En ce moment, Aniss saisit le sac bleu.
+narrateur|Le tissu gratte sous ses doigts.
+papa|Prends de l'eau, pour le chemin.
+narrateur|Aniss prend la gourde fraîche.
+narrateur|Le bouchon est froid sous le doigt.
 papa|Le chapeau aussi, les branches piquent.
-narrateur|Aniss prend le chapeau.
-narrateur|Le bord est un peu souple.
-narrateur|Le chapeau glisse par terre.
-enfant-m|Il est tombé.
-papa|Tu le ramasses, puis dans le sac.
-narrateur|Aniss ramasse le chapeau.
-narrateur|Il le met dans le sac.
-enfant-m|Et le doudou ?
-narrateur|Le doudou n'est pas près des chaussures.
-papa|Regarde la chaise de la cuisine.</t>
+narrateur|Aniss prend le chapeau souple.
+narrateur|Le bord plie un peu, dans sa main.
+enfant-m|Et ma boîte à plumes ?
+narrateur|La boîte de bois attend sur le banc.
+enfant-m|Je mets tout, d'un coup !
+narrateur|Il pousse gourde, chapeau et boîte.
+narrateur|La boîte tape le fond, trop vite.
+narrateur|Le zip mord le bord du chapeau.
+enfant-m|Ça reste coincé !
+narrateur|Le sourire d'Aniss disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+papa|Tu regardes le zip ?</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>oiseau</t>
+          <t>pin,vitre,sac</t>
         </is>
       </c>
     </row>
@@ -1396,12 +1400,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Aniss prépare le sac. Où met-il les affaires ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Aniss prépare le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;. Où met-il les affaires ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Clara prépare le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Que met-elle ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Aniss prépare le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Où met-il les affaires ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1464,7 +1468,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1475,7 +1479,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1490,11 +1494,11 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
@@ -1505,23 +1509,23 @@
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1536,17 +1540,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=les_affaires_vont_dans_le_sac; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1579,17 +1583,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Le doudou est sur la chaise de la cuisine. Il sent le coton. Il est tout doux. Aniss le met dans le sac. Te voilà. Merci, Aniss. Aniss ferme le sac. Ça fait zzz. Il le porte. Le sac est prêt ? Oui, papa. La sangle n'est plus froide. Tu as fini ta tartine ? Oui, papa. Alors on va voir l'oiseau. Une miette reste près de la tasse. On la laisse pour plus tard.</t>
+          <t>Papa s'accroupit à la même hauteur. Aniss refuse de tirer plus fort. Je sors le chapeau. Il tire le tissu coincé, sans forcer. Le zip lâche, petit à petit. Il pose le chapeau à plat, sur la table. L'eau va au fond. Aniss range la gourde froide. La boîte de bois glisse à côté. Et mon doudou ? Le doudou n'est pas près des chaussures. Regarde le banc sous la fenêtre. Aniss cherche près du banc. Le doudou sent le coton, un peu chaud. Te voilà. Il le glisse dans le sac. Merci, Aniss. Le zip avance, sans mordre. Il part. Le sac est prêt ? Pas le grain. Tu prends aussi le grain de pin ? Oui, pour la plume. Aniss détache le grain de la vitre. Il le pose dans la boîte de bois. Aniss appuie sur la fermeture. Ça fait un petit zzz. Le sac bleu est fermé.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Le doudou est sur la chaise de la cuisine. Il sent le coton. Il est tout doux. Aniss le met dans le sac. Te voilà. Merci, Aniss. Aniss ferme le sac. Ça fait zzz. Il le porte. Le sac est prêt ? Oui, papa. La sangle n'est plus froide. Tu as fini ta tartine ? Oui, papa. Alors on va voir l'oiseau. Une miette reste près de la tasse. On la laisse pour plus tard.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Papa s'accroupit à la même hauteur. Aniss refuse de tirer plus fort. Je sors le chapeau. Il tire le tissu coincé, sans forcer. Le zip lâche, petit à petit. Il pose le chapeau à plat, sur la table. L'eau va au fond. Aniss range la gourde froide. La boîte de bois glisse à côté. Et mon doudou ? Le doudou n'est pas près des chaussures. Regarde le banc sous la fenêtre. Aniss cherche près du banc. Le doudou sent le coton, un peu chaud. Te voilà. Il le glisse dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;. Merci, Aniss. Le zip avance, sans mordre. Il part. Le sac est prêt ? Pas le grain. Tu prends aussi le grain de pin ? Oui, pour la plume. Aniss détache le grain de la vitre. Il le pose dans la boîte de bois. Aniss appuie sur la fermeture. Ça fait un petit zzz. Le sac bleu est fermé.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Clara a préparé son &lt;emphasis&gt;sac&lt;/emphasis&gt;. Elle a mis ce que l'adulte a dit. Papa était là. [pause]</t>
+          <t>Papa s'accroupit à la même hauteur. Aniss refuse de tirer plus fort. Je sors le chapeau. Il tire le tissu coincé, sans forcer. Le zip lâche, petit à petit. Il pose le chapeau à plat, sur la table. L'eau va au fond. Aniss range la gourde froide. La boîte de bois glisse à côté. Et mon doudou ? Le doudou n'est pas près des chaussures. Regarde le banc sous la fenêtre. Aniss cherche près du banc. Le doudou sent le coton, un peu chaud. Te voilà. Il le glisse dans le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Merci, Aniss. Le zip avance, sans mordre. Il part. Le sac est prêt ? Pas le grain. Tu prends aussi le grain de pin ? Oui, pour la plume. Aniss détache le grain de la vitre. Il le pose dans la boîte de bois. Aniss appuie sur la fermeture. Ça fait un petit zzz. Le sac bleu est fermé. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1647,7 +1651,7 @@
         <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1684,16 +1688,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1718,28 +1722,44 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=faire_vivre_le_geste; emotion=concentration puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=une_chose_puis_la_suivante; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Le doudou est sur la chaise de la cuisine.
-narrateur|Il sent le coton.
-narrateur|Il est tout doux.
-narrateur|Aniss le met dans le sac.
+          <t>narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Aniss refuse de tirer plus fort.
+enfant-m|Je sors le chapeau.
+narrateur|Il tire le tissu coincé, sans forcer.
+narrateur|Le zip lâche, petit à petit.
+narrateur|Il pose le chapeau à plat, sur la table.
+papa|L'eau va au fond.
+narrateur|Aniss range la gourde froide.
+narrateur|La boîte de bois glisse à côté.
+enfant-m|Et mon doudou ?
+narrateur|Le doudou n'est pas près des chaussures.
+papa|Regarde le banc sous la fenêtre.
+narrateur|Aniss cherche près du banc.
+narrateur|Le doudou sent le coton, un peu chaud.
 enfant-m|Te voilà.
+narrateur|Il le glisse dans le sac.
 papa|Merci, Aniss.
-narrateur|Aniss ferme le sac.
-narrateur|Ça fait zzz.
-narrateur|Il le porte.
+narrateur|Le zip avance, sans mordre.
+enfant-m|Il part.
 papa|Le sac est prêt ?
-enfant-m|Oui, papa.
-narrateur|La sangle n'est plus froide.
-papa|Tu as fini ta tartine ?
-enfant-m|Oui, papa.
-papa|Alors on va voir l'oiseau.
-narrateur|Une miette reste près de la tasse.
-papa|On la laisse pour plus tard.</t>
+enfant-m|Pas le grain.
+papa|Tu prends aussi le grain de pin ?
+enfant-m|Oui, pour la plume.
+narrateur|Aniss détache le grain de la vitre.
+narrateur|Il le pose dans la boîte de bois.
+narrateur|Aniss appuie sur la fermeture.
+narrateur|Ça fait un petit zzz.
+narrateur|Le sac bleu est fermé.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>zip,tissu</t>
         </is>
       </c>
     </row>
@@ -1766,17 +1786,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On met tes chaussures. Aniss enfile ses chaussures. Tu as fini tes chaussures ? Oui, papa. On ouvre la porte. Papa ouvre la porte. L'air sent le pin et l'herbe sèche. L'oiseau chante encore. Je l'entends, papa. Oui, il est dans le grand arbre. Ils marchent sur le chemin du bois. Le sac tape doucement. La tartine n'est plus sur l'assiette. Ils s'arrêtent sous le grand arbre. Une feuille bouge. Il est là-haut. Oui, on écoute encore un peu. L'oiseau fait un petit cri. Aniss lève le menton. Une plume grise est dans l'herbe. Pour moi ? Tu la prends tout doux ? Aniss ramasse la plume. Elle est légère, presque rien.</t>
+          <t>On met tes chaussures ? Aniss enfile ses chaussures. Une semelle est froide, contre le sol. Tu as fini tes chaussures ? Oui, papa. On ouvre la porte. Papa ouvre la porte. L'air sent la résine et l'herbe sèche. Le sac bleu tape contre sa hanche. On va voir la plume ? Oui, sous le grand arbre. Ils marchent sur le chemin du bois. Les aiguilles de pin craquent sous les pas. Je la vois, papa ! Une plume grise brille, plus loin. Je cours la prendre ! Aniss veut partir sans le sac. Une branche basse barre le pas. Le sourire d'Aniss se serre. Ça serre, dans son ventre. Je n'aime pas ça. Aniss refuse de foncer. Attends, je regarde. Personne ne donne la réponse. Aniss observe le sac, écoute le bois. Dans la boîte, le grain de pin a bougé. Il penche vers la branche basse. C'est par là. Tu contournes, ou tu pousses ? Je contourne. Il recule d'un pas. Il passe sous la branche, lentement. Le sac reste bien fermé. Elle est là. Oui, dans l'herbe.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>On met tes chaussures. Aniss enfile ses chaussures. Tu as fini tes chaussures ? Oui, papa. On ouvre la porte. Papa ouvre la porte. L'air sent le pin et l'herbe sèche. L'oiseau chante encore. Je l'entends, papa. Oui, il est dans le grand arbre. Ils marchent sur le chemin du bois. Le sac tape doucement. La tartine n'est plus sur l'assiette. Ils s'arrêtent sous le grand arbre. Une feuille bouge. Il est là-haut. Oui, on écoute encore un peu. L'oiseau fait un petit cri. Aniss lève le menton. Une plume grise est dans l'herbe. Pour moi ? Tu la prends tout doux ? Aniss ramasse la plume. Elle est légère, presque rien.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On met tes chaussures ? Aniss enfile ses chaussures. Une semelle est froide, contre le sol. Tu as fini tes chaussures ? Oui, papa. On ouvre la porte. Papa ouvre la porte. L'air sent la résine et l'herbe sèche. Le sac bleu tape contre sa hanche. On va voir la plume ? Oui, sous le grand arbre. Ils marchent sur le chemin du bois. Les aiguilles de pin craquent sous les pas. Je la vois, papa ! Une plume grise brille, plus loin. Je cours la prendre ! Aniss veut partir sans le sac. Une branche basse barre le pas. Le sourire d'Aniss se serre. Ça serre, dans son ventre. Je n'aime pas ça. Aniss refuse de foncer. Attends, je regarde. Personne ne donne la réponse. Aniss observe le sac, écoute le bois. Dans la boîte, le &lt;emphasis level="moderate"&gt;grain de pin&lt;/emphasis&gt; a bougé. Il penche vers la branche basse. C'est par là. Tu contournes, ou tu pousses ? Je contourne. Il recule d'un pas. Il passe sous la branche, lentement. Le sac reste bien fermé. Elle est là. Oui, dans l'herbe.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Clara porte le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Papa ouvre la porte. [pause]</t>
+          <t>On met tes chaussures ? Aniss enfile ses chaussures. Une semelle est froide, contre le sol. Tu as fini tes chaussures ? Oui, papa. On ouvre la porte. Papa ouvre la porte. L'air sent la résine et l'herbe sèche. Le sac bleu tape contre sa hanche. On va voir la plume ? Oui, sous le grand arbre. Ils marchent sur le chemin du bois. Les aiguilles de pin craquent sous les pas. Je la vois, papa ! Une plume grise brille, plus loin. Je cours la prendre ! Aniss veut partir sans le sac. Une branche basse barre le pas. Le sourire d'Aniss se serre. Ça serre, dans son ventre. Je n'aime pas ça. Aniss refuse de foncer. Attends, je regarde. Personne ne donne la réponse. Aniss observe le sac, écoute le bois. Dans la boîte, le &lt;emphasis&gt;grain de pin&lt;/emphasis&gt; a bougé. Il penche vers la branche basse. C'est par là. Tu contournes, ou tu pousses ? Je contourne. Il recule d'un pas. Il passe sous la branche, lentement. Le sac reste bien fermé. Elle est là. Oui, dans l'herbe. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1823,7 +1843,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1831,10 +1851,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1857,30 +1877,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>sac</t>
+          <t>grain de pin</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1889,10 +1909,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1903,33 +1923,53 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_sous_la_branche; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>papa|On met tes chaussures.
+          <t>papa|On met tes chaussures ?
 narrateur|Aniss enfile ses chaussures.
+narrateur|Une semelle est froide, contre le sol.
 papa|Tu as fini tes chaussures ?
 enfant-m|Oui, papa.
 papa|On ouvre la porte.
 narrateur|Papa ouvre la porte.
-narrateur|L'air sent le pin et l'herbe sèche.
-narrateur|L'oiseau chante encore.
-enfant-m|Je l'entends, papa.
-papa|Oui, il est dans le grand arbre.
+narrateur|L'air sent la résine et l'herbe sèche.
+narrateur|Le sac bleu tape contre sa hanche.
+enfant-m|On va voir la plume ?
+papa|Oui, sous le grand arbre.
 narrateur|Ils marchent sur le chemin du bois.
-narrateur|Le sac tape doucement.
-narrateur|La tartine n'est plus sur l'assiette.
-narrateur|Ils s'arrêtent sous le grand arbre.
-narrateur|Une feuille bouge.
-enfant-m|Il est là-haut.
-papa|Oui, on écoute encore un peu.
-narrateur|L'oiseau fait un petit cri.
-narrateur|Aniss lève le menton.
-narrateur|Une plume grise est dans l'herbe.
-enfant-m|Pour moi ?
-papa|Tu la prends tout doux ?
-narrateur|Aniss ramasse la plume.
-narrateur|Elle est légère, presque rien.</t>
+narrateur|Les aiguilles de pin craquent sous les pas.
+enfant-m|Je la vois, papa !
+narrateur|Une plume grise brille, plus loin.
+enfant-m|Je cours la prendre !
+narrateur|Aniss veut partir sans le sac.
+narrateur|Une branche basse barre le pas.
+narrateur|Le sourire d'Aniss se serre.
+narrateur|Ça serre, dans son ventre.
+enfant-m|Je n'aime pas ça.
+narrateur|Aniss refuse de foncer.
+enfant-m|Attends, je regarde.
+narrateur|Personne ne donne la réponse.
+narrateur|Aniss observe le sac, écoute le bois.
+narrateur|Dans la boîte, le grain de pin a bougé.
+narrateur|Il penche vers la branche basse.
+enfant-m|C'est par là.
+papa|Tu contournes, ou tu pousses ?
+enfant-m|Je contourne.
+narrateur|Il recule d'un pas.
+narrateur|Il passe sous la branche, lentement.
+narrateur|Le sac reste bien fermé.
+enfant-m|Elle est là.
+papa|Oui, dans l'herbe.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>chemin,branches</t>
         </is>
       </c>
     </row>
@@ -1956,17 +1996,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>La plume chatouille le doigt d'Aniss. L'oiseau chante plus fort. On l'a vu. On l'a entendu. Le sac voyage sur le dos d'Aniss. Les aiguilles de pin sentent encore le chaud. Le doudou est chaud, contre toi. Aniss reste un moment, tout calme, sous l'arbre.</t>
+          <t>Ils s'arrêtent sous le grand arbre. L'ombre de l'arbre touche les joues d'Aniss. La plume est là. Oui, elle t'attendait. Une plume grise repose dans l'herbe sèche. Sur la plume, un grain de pin brille. Comme sur la vitre, papa ! Tu la prends, toi ? Oui, dans ma boîte. Aniss ouvre le sac, sans se presser. Il glisse la plume contre le grain de pin. Le grain colle un peu à la plume. Ils voyagent ensemble. Tu les sens, sur tes doigts ? Oui, ça sent le bois. Le sac repose contre sa hanche. Le grain de pin brille sur la plume.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>La plume chatouille le doigt d'Aniss. L'oiseau chante plus fort. On l'a vu. On l'a entendu. Le sac voyage sur le dos d'Aniss. Les aiguilles de pin sentent encore le chaud. Le doudou est chaud, contre toi. Aniss reste un moment, tout calme, sous l'arbre.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils s'arrêtent sous le grand arbre. L'ombre de l'arbre touche les joues d'Aniss. La plume est là. Oui, elle t'attendait. Une plume grise repose dans l'herbe sèche. Sur la plume, un &lt;emphasis level="moderate"&gt;grain de pin&lt;/emphasis&gt; brille. Comme sur la vitre, papa ! Tu la prends, toi ? Oui, dans ma boîte. Aniss ouvre le sac, sans se presser. Il glisse la plume contre le grain de pin. Le grain colle un peu à la plume. Ils voyagent ensemble. Tu les sens, sur tes doigts ? Oui, ça sent le bois. Le sac repose contre sa hanche. Le grain de pin brille sur la plume.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils s'arrêtent sous le grand arbre. L'ombre de l'arbre touche les joues d'Aniss. La plume est là. Oui, elle t'attendait. Une plume grise repose dans l'herbe sèche. Sur la plume, un &lt;emphasis&gt;grain de pin&lt;/emphasis&gt; brille. Comme sur la vitre, papa ! Tu la prends, toi ? Oui, dans ma boîte. Aniss ouvre le sac, sans se presser. Il glisse la plume contre le grain de pin. Le grain colle un peu à la plume. Ils voyagent ensemble. Tu les sens, sur tes doigts ? Oui, ça sent le bois. Le sac repose contre sa hanche. Le grain de pin brille sur la plume.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2013,18 +2053,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2033,12 +2073,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2047,17 +2087,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>grain de pin</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2066,11 +2110,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2079,31 +2123,49 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=le_grain_de_la_vitre_est_sur_la_plume; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|La plume chatouille le doigt d'Aniss.
-narrateur|L'oiseau chante plus fort.
-enfant-m|On l'a vu.
-papa|On l'a entendu.
-narrateur|Le sac voyage sur le dos d'Aniss.
-narrateur|Les aiguilles de pin sentent encore le chaud.
-papa|Le doudou est chaud, contre toi.
-narrateur|Aniss reste un moment, tout calme, sous l'arbre.</t>
+          <t>narrateur|Ils s'arrêtent sous le grand arbre.
+narrateur|L'ombre de l'arbre touche les joues d'Aniss.
+enfant-m|La plume est là.
+papa|Oui, elle t'attendait.
+narrateur|Une plume grise repose dans l'herbe sèche.
+narrateur|Sur la plume, un grain de pin brille.
+enfant-m|Comme sur la vitre, papa !
+papa|Tu la prends, toi ?
+enfant-m|Oui, dans ma boîte.
+narrateur|Aniss ouvre le sac, sans se presser.
+narrateur|Il glisse la plume contre le grain de pin.
+narrateur|Le grain colle un peu à la plume.
+enfant-m|Ils voyagent ensemble.
+papa|Tu les sens, sur tes doigts ?
+enfant-m|Oui, ça sent le bois.
+narrateur|Le sac repose contre sa hanche.
+narrateur|Le grain de pin brille sur la plume.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>arbre,plume</t>
         </is>
       </c>
     </row>
@@ -2124,7 +2186,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2216,6 +2278,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>